<commit_message>
Checkpoint before assistant change: Add NIRF data from Excel file.
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/attached_assets/Copy of nirf_tables(1).xlsx
+++ b/attached_assets/Copy of nirf_tables(1).xlsx
@@ -1,26 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nihal\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0e021ffd7526bcf4/NIRF1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{87B7B011-6721-463A-98CC-DBCCE7692EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_8D8119E0C643DF22856E482A9C109B2B486D3750" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6EDF1912-5CE2-463F-B27D-5B9E3CC33E79}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2024" sheetId="1" r:id="rId1"/>
+    <sheet name="Top 10 Autonomous" sheetId="2" r:id="rId2"/>
+    <sheet name="Top 10 Telangana" sheetId="3" r:id="rId3"/>
+    <sheet name="Top 10 Telangana Autonomous" sheetId="4" r:id="rId4"/>
+    <sheet name="Top 10 South India" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="138">
   <si>
     <t>S.no</t>
   </si>
@@ -118,6 +122,9 @@
     <t>S.R.M. Institute of Science and Technology</t>
   </si>
   <si>
+    <t>Anna University</t>
+  </si>
+  <si>
     <t>Indian Institute of Technology (Indian School of Mines) Dhanbad</t>
   </si>
   <si>
@@ -160,12 +167,18 @@
     <t>Indian Institute of Technology Jodhpur</t>
   </si>
   <si>
+    <t>Thappar Institute of Engineering and Technology</t>
+  </si>
+  <si>
     <t>Amity University</t>
   </si>
   <si>
     <t>Indian Institute of Technology Mandi</t>
   </si>
   <si>
+    <t>Chandigarh University</t>
+  </si>
+  <si>
     <t>Aligarh Muslim University</t>
   </si>
   <si>
@@ -208,6 +221,9 @@
     <t>Sri Sivasubramaniya Nadar College of Engineering</t>
   </si>
   <si>
+    <t>722:</t>
+  </si>
+  <si>
     <t>Technology Hyderabad</t>
   </si>
   <si>
@@ -220,9 +236,15 @@
     <t>Lovely Professional University</t>
   </si>
   <si>
+    <t>TAL</t>
+  </si>
+  <si>
     <t>Indian Institute of Space Science and Technology</t>
   </si>
   <si>
+    <t>Graphic Era University</t>
+  </si>
+  <si>
     <t>Saveetha Institute of Medical and Technical Sciences</t>
   </si>
   <si>
@@ -247,6 +269,9 @@
     <t>Motilal Nehru National Institute of Technology</t>
   </si>
   <si>
+    <t>B41</t>
+  </si>
+  <si>
     <t>Indian Institute of Technology Tirupati</t>
   </si>
   <si>
@@ -286,6 +311,9 @@
     <t>Indian Institute of Technology Bhilai</t>
   </si>
   <si>
+    <t>7A2</t>
+  </si>
+  <si>
     <t>International Institute of Information Technology Bangalore</t>
   </si>
   <si>
@@ -337,12 +365,18 @@
     <t>AU College of Engineering</t>
   </si>
   <si>
+    <t>TIT</t>
+  </si>
+  <si>
     <t>ce, Technology and Research</t>
   </si>
   <si>
     <t>technology and Management Sciences</t>
   </si>
   <si>
+    <t>B44</t>
+  </si>
+  <si>
     <t>Christ University</t>
   </si>
   <si>
@@ -361,47 +395,56 @@
     <t>SR University</t>
   </si>
   <si>
+    <t>R.V College of Engineering</t>
+  </si>
+  <si>
     <t>Siddaganga Institute of Technology</t>
   </si>
   <si>
-    <t>TAL</t>
-  </si>
-  <si>
-    <t>B41</t>
-  </si>
-  <si>
-    <t>B44</t>
-  </si>
-  <si>
-    <t>722:</t>
-  </si>
-  <si>
-    <t>7A2</t>
-  </si>
-  <si>
-    <t>TIT</t>
-  </si>
-  <si>
-    <t>Anna University</t>
-  </si>
-  <si>
-    <t>Thappar Institute of Engineering and Technology</t>
-  </si>
-  <si>
-    <t>Chandigarh University</t>
-  </si>
-  <si>
-    <t>Graphic Era University</t>
-  </si>
-  <si>
-    <t>R.V College of Engineering</t>
+    <t>International Institute of Information Technology Hyderabad</t>
+  </si>
+  <si>
+    <t>Goka Raju Ranga Raju Institute of Engineering &amp; Technology</t>
+  </si>
+  <si>
+    <t>Mahindra University</t>
+  </si>
+  <si>
+    <t>University College of Engineering</t>
+  </si>
+  <si>
+    <t>Anurag University</t>
+  </si>
+  <si>
+    <t>Chaitanya Bharathi Institute of Technology</t>
+  </si>
+  <si>
+    <t>CVR College of Engineering</t>
+  </si>
+  <si>
+    <t>Institute of Aeronautical Engineering</t>
+  </si>
+  <si>
+    <t>Maulana Azad National Urdu University</t>
+  </si>
+  <si>
+    <t>Chennai Institute of Technology</t>
+  </si>
+  <si>
+    <t>Coimbatore Institute of Technology</t>
+  </si>
+  <si>
+    <t>College of Engineering, Trivandrum</t>
+  </si>
+  <si>
+    <t>Gandhi Institute of Technology and Management</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,6 +460,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -426,7 +474,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -449,15 +497,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1599,7 +1685,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>120</v>
+        <v>32</v>
       </c>
       <c r="C15">
         <v>15.94</v>
@@ -1658,7 +1744,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C16">
         <v>15.43</v>
@@ -1717,7 +1803,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C17">
         <v>10.73</v>
@@ -1776,7 +1862,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C18">
         <v>17.5</v>
@@ -1835,7 +1921,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C19">
         <v>11.5</v>
@@ -1894,7 +1980,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C20">
         <v>17.5</v>
@@ -1953,7 +2039,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C21">
         <v>17.87</v>
@@ -2012,7 +2098,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C22">
         <v>16.5</v>
@@ -2071,7 +2157,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C23">
         <v>1241</v>
@@ -2130,7 +2216,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C24">
         <v>16.22</v>
@@ -2189,7 +2275,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C25">
         <v>10.5</v>
@@ -2248,7 +2334,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C26">
         <v>16</v>
@@ -2307,7 +2393,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C27">
         <v>17.5</v>
@@ -2366,7 +2452,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C28">
         <v>19</v>
@@ -2425,7 +2511,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C29">
         <v>12.53</v>
@@ -2484,7 +2570,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>121</v>
+        <v>47</v>
       </c>
       <c r="C30">
         <v>18.23</v>
@@ -2543,7 +2629,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C31">
         <v>16.47</v>
@@ -2602,7 +2688,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C32">
         <v>9.7899999999999991</v>
@@ -2661,7 +2747,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>122</v>
+        <v>50</v>
       </c>
       <c r="C33">
         <v>17.95</v>
@@ -2720,7 +2806,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C34">
         <v>11</v>
@@ -2779,7 +2865,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C35">
         <v>12.02</v>
@@ -2838,7 +2924,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C36">
         <v>1747</v>
@@ -2897,7 +2983,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C37">
         <v>16.48</v>
@@ -2956,7 +3042,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C38">
         <v>20</v>
@@ -3015,7 +3101,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C39">
         <v>16.32</v>
@@ -3074,7 +3160,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C40">
         <v>13.94</v>
@@ -3133,7 +3219,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C41">
         <v>14.35</v>
@@ -3192,7 +3278,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C42">
         <v>1037</v>
@@ -3251,7 +3337,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C43">
         <v>15.5</v>
@@ -3310,7 +3396,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C44">
         <v>14.97</v>
@@ -3369,7 +3455,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C45">
         <v>14.09</v>
@@ -3428,7 +3514,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C46">
         <v>7.96</v>
@@ -3487,7 +3573,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C47">
         <v>13.5</v>
@@ -3532,7 +3618,7 @@
         <v>25.67</v>
       </c>
       <c r="Q47" t="s">
-        <v>117</v>
+        <v>65</v>
       </c>
       <c r="R47">
         <v>20</v>
@@ -3546,7 +3632,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C48">
         <v>9.33</v>
@@ -3605,7 +3691,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C49">
         <v>13.49</v>
@@ -3664,7 +3750,7 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C50">
         <v>12.26</v>
@@ -3723,7 +3809,7 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C51">
         <v>18</v>
@@ -3735,7 +3821,7 @@
         <v>12.22</v>
       </c>
       <c r="F51" t="s">
-        <v>114</v>
+        <v>70</v>
       </c>
       <c r="G51">
         <v>16.53</v>
@@ -3782,7 +3868,7 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C52">
         <v>8.9499999999999993</v>
@@ -3841,7 +3927,7 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>123</v>
+        <v>72</v>
       </c>
       <c r="C53">
         <v>12.7</v>
@@ -3900,7 +3986,7 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C54">
         <v>13.18</v>
@@ -3959,7 +4045,7 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C55">
         <v>11.15</v>
@@ -4018,7 +4104,7 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C56">
         <v>12.35</v>
@@ -4077,7 +4163,7 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C57">
         <v>15.12</v>
@@ -4136,7 +4222,7 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C58">
         <v>15.04</v>
@@ -4195,7 +4281,7 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="C59">
         <v>14.1</v>
@@ -4254,7 +4340,7 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C60">
         <v>12.96</v>
@@ -4313,7 +4399,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C61">
         <v>16.010000000000002</v>
@@ -4358,7 +4444,7 @@
         <v>1145</v>
       </c>
       <c r="Q61" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
       <c r="R61">
         <v>20</v>
@@ -4372,7 +4458,7 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C62">
         <v>8.32</v>
@@ -4431,7 +4517,7 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="C63">
         <v>798</v>
@@ -4490,7 +4576,7 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C64">
         <v>4.8600000000000003</v>
@@ -4549,7 +4635,7 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C65">
         <v>14.6</v>
@@ -4608,7 +4694,7 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="C66">
         <v>14.67</v>
@@ -4667,7 +4753,7 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C67">
         <v>16.53</v>
@@ -4726,7 +4812,7 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="C68">
         <v>14.62</v>
@@ -4785,7 +4871,7 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C69">
         <v>6.64</v>
@@ -4844,7 +4930,7 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C70">
         <v>727</v>
@@ -4903,7 +4989,7 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C71">
         <v>4.9000000000000004</v>
@@ -4933,7 +5019,7 @@
         <v>18.22</v>
       </c>
       <c r="L71" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
       <c r="M71">
         <v>12.18</v>
@@ -4962,7 +5048,7 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C72">
         <v>13.94</v>
@@ -5021,7 +5107,7 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C73">
         <v>15.01</v>
@@ -5080,7 +5166,7 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="C74">
         <v>6.36</v>
@@ -5125,7 +5211,7 @@
         <v>9.2200000000000006</v>
       </c>
       <c r="Q74" t="s">
-        <v>118</v>
+        <v>95</v>
       </c>
       <c r="R74">
         <v>20</v>
@@ -5139,7 +5225,7 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="C75">
         <v>843</v>
@@ -5198,7 +5284,7 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="C76">
         <v>14.4</v>
@@ -5257,7 +5343,7 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="C77">
         <v>10</v>
@@ -5316,7 +5402,7 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C78">
         <v>11.5</v>
@@ -5375,7 +5461,7 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="C79">
         <v>10.68</v>
@@ -5434,7 +5520,7 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="C80">
         <v>12.79</v>
@@ -5493,7 +5579,7 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C81">
         <v>8</v>
@@ -5552,7 +5638,7 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="C82">
         <v>14.63</v>
@@ -5611,7 +5697,7 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="C83">
         <v>12.59</v>
@@ -5670,7 +5756,7 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="C84">
         <v>13.5</v>
@@ -5729,7 +5815,7 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C85">
         <v>13.22</v>
@@ -5788,7 +5874,7 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="C86">
         <v>11.7</v>
@@ -5847,7 +5933,7 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="C87">
         <v>15.13</v>
@@ -5906,7 +5992,7 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="C88">
         <v>10.54</v>
@@ -5965,7 +6051,7 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C89">
         <v>14.5</v>
@@ -6024,7 +6110,7 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C90">
         <v>11</v>
@@ -6083,7 +6169,7 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="C91">
         <v>11.49</v>
@@ -6128,7 +6214,7 @@
         <v>30</v>
       </c>
       <c r="Q91" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="R91">
         <v>20</v>
@@ -6142,7 +6228,7 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="C92">
         <v>14.65</v>
@@ -6201,7 +6287,7 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="C93">
         <v>9.0399999999999991</v>
@@ -6260,7 +6346,7 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="C94">
         <v>8.26</v>
@@ -6319,7 +6405,7 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="C95">
         <v>15.47</v>
@@ -6378,7 +6464,7 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="C96">
         <v>13.23</v>
@@ -6437,7 +6523,7 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="C97">
         <v>15.38</v>
@@ -6496,7 +6582,7 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="C98">
         <v>8.9700000000000006</v>
@@ -6555,7 +6641,7 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="C99">
         <v>13.97</v>
@@ -6614,7 +6700,7 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C100">
         <v>14</v>
@@ -6673,7 +6759,7 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="C101">
         <v>12.42</v>
@@ -6725,6 +6811,1006 @@
       </c>
       <c r="S101">
         <v>10.06</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="66.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2">
+        <v>18.5</v>
+      </c>
+      <c r="D2">
+        <v>30</v>
+      </c>
+      <c r="E2">
+        <v>17.29</v>
+      </c>
+      <c r="F2">
+        <v>30</v>
+      </c>
+      <c r="G2">
+        <v>34.950000000000003</v>
+      </c>
+      <c r="H2">
+        <v>34.369999999999997</v>
+      </c>
+      <c r="I2">
+        <v>14</v>
+      </c>
+      <c r="J2">
+        <v>978</v>
+      </c>
+      <c r="K2">
+        <v>29.74</v>
+      </c>
+      <c r="L2">
+        <v>15</v>
+      </c>
+      <c r="M2">
+        <v>19.34</v>
+      </c>
+      <c r="N2">
+        <v>16.98</v>
+      </c>
+      <c r="O2">
+        <v>21.57</v>
+      </c>
+      <c r="P2">
+        <v>14.88</v>
+      </c>
+      <c r="Q2">
+        <v>9.4</v>
+      </c>
+      <c r="R2">
+        <v>20</v>
+      </c>
+      <c r="S2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>18.5</v>
+      </c>
+      <c r="D3">
+        <v>23.18</v>
+      </c>
+      <c r="E3">
+        <v>15.61</v>
+      </c>
+      <c r="F3">
+        <v>2841</v>
+      </c>
+      <c r="G3">
+        <v>35</v>
+      </c>
+      <c r="H3">
+        <v>37.630000000000003</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
+      </c>
+      <c r="J3">
+        <v>6.56</v>
+      </c>
+      <c r="K3">
+        <v>33.049999999999997</v>
+      </c>
+      <c r="L3">
+        <v>13.06</v>
+      </c>
+      <c r="M3">
+        <v>20.93</v>
+      </c>
+      <c r="N3">
+        <v>17.489999999999998</v>
+      </c>
+      <c r="O3">
+        <v>24.05</v>
+      </c>
+      <c r="P3">
+        <v>14.07</v>
+      </c>
+      <c r="Q3">
+        <v>727</v>
+      </c>
+      <c r="R3">
+        <v>20</v>
+      </c>
+      <c r="S3">
+        <v>98.53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4">
+        <v>18.329999999999998</v>
+      </c>
+      <c r="D4">
+        <v>28.72</v>
+      </c>
+      <c r="E4">
+        <v>19.45</v>
+      </c>
+      <c r="F4">
+        <v>27.76</v>
+      </c>
+      <c r="G4">
+        <v>28.49</v>
+      </c>
+      <c r="H4">
+        <v>28.87</v>
+      </c>
+      <c r="I4">
+        <v>10</v>
+      </c>
+      <c r="J4">
+        <v>6.72</v>
+      </c>
+      <c r="K4">
+        <v>36.130000000000003</v>
+      </c>
+      <c r="L4">
+        <v>15</v>
+      </c>
+      <c r="M4">
+        <v>21.84</v>
+      </c>
+      <c r="N4">
+        <v>16.079999999999998</v>
+      </c>
+      <c r="O4">
+        <v>19.940000000000001</v>
+      </c>
+      <c r="P4">
+        <v>12.94</v>
+      </c>
+      <c r="Q4">
+        <v>774</v>
+      </c>
+      <c r="R4">
+        <v>20</v>
+      </c>
+      <c r="S4">
+        <v>84.19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5">
+        <v>19.760000000000002</v>
+      </c>
+      <c r="D5">
+        <v>21.5</v>
+      </c>
+      <c r="E5">
+        <v>14.79</v>
+      </c>
+      <c r="F5">
+        <v>22.47</v>
+      </c>
+      <c r="G5">
+        <v>30.68</v>
+      </c>
+      <c r="H5">
+        <v>34.86</v>
+      </c>
+      <c r="I5">
+        <v>10</v>
+      </c>
+      <c r="J5">
+        <v>3.75</v>
+      </c>
+      <c r="K5">
+        <v>24.3</v>
+      </c>
+      <c r="L5">
+        <v>13.99</v>
+      </c>
+      <c r="M5">
+        <v>20.87</v>
+      </c>
+      <c r="N5">
+        <v>20</v>
+      </c>
+      <c r="O5">
+        <v>21.87</v>
+      </c>
+      <c r="P5">
+        <v>11.93</v>
+      </c>
+      <c r="Q5">
+        <v>4.0199999999999996</v>
+      </c>
+      <c r="R5">
+        <v>20</v>
+      </c>
+      <c r="S5">
+        <v>80.260000000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6">
+        <v>17.66</v>
+      </c>
+      <c r="D6">
+        <v>23.13</v>
+      </c>
+      <c r="E6">
+        <v>15.28</v>
+      </c>
+      <c r="F6">
+        <v>21.67</v>
+      </c>
+      <c r="G6">
+        <v>30.25</v>
+      </c>
+      <c r="H6">
+        <v>33.200000000000003</v>
+      </c>
+      <c r="I6">
+        <v>7</v>
+      </c>
+      <c r="J6">
+        <v>425</v>
+      </c>
+      <c r="K6">
+        <v>37.74</v>
+      </c>
+      <c r="L6">
+        <v>15</v>
+      </c>
+      <c r="M6">
+        <v>20.170000000000002</v>
+      </c>
+      <c r="N6">
+        <v>14.44</v>
+      </c>
+      <c r="O6">
+        <v>23.72</v>
+      </c>
+      <c r="P6">
+        <v>12.64</v>
+      </c>
+      <c r="Q6">
+        <v>5.84</v>
+      </c>
+      <c r="R6">
+        <v>20</v>
+      </c>
+      <c r="S6">
+        <v>65.790000000000006</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7">
+        <v>18.32</v>
+      </c>
+      <c r="D7">
+        <v>24.57</v>
+      </c>
+      <c r="E7">
+        <v>13.71</v>
+      </c>
+      <c r="F7">
+        <v>20.22</v>
+      </c>
+      <c r="G7">
+        <v>29.8</v>
+      </c>
+      <c r="H7">
+        <v>29.68</v>
+      </c>
+      <c r="I7">
+        <v>3</v>
+      </c>
+      <c r="J7">
+        <v>5.58</v>
+      </c>
+      <c r="K7">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="L7">
+        <v>14.94</v>
+      </c>
+      <c r="M7">
+        <v>21.63</v>
+      </c>
+      <c r="N7">
+        <v>15.71</v>
+      </c>
+      <c r="O7">
+        <v>24.79</v>
+      </c>
+      <c r="P7">
+        <v>11.94</v>
+      </c>
+      <c r="Q7">
+        <v>2.84</v>
+      </c>
+      <c r="R7">
+        <v>20</v>
+      </c>
+      <c r="S7">
+        <v>55.38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8">
+        <v>1241</v>
+      </c>
+      <c r="D8">
+        <v>30</v>
+      </c>
+      <c r="E8">
+        <v>19.489999999999998</v>
+      </c>
+      <c r="F8">
+        <v>26.83</v>
+      </c>
+      <c r="G8">
+        <v>25.51</v>
+      </c>
+      <c r="H8">
+        <v>23.82</v>
+      </c>
+      <c r="I8">
+        <v>3</v>
+      </c>
+      <c r="J8">
+        <v>5.18</v>
+      </c>
+      <c r="K8">
+        <v>33.08</v>
+      </c>
+      <c r="L8">
+        <v>15</v>
+      </c>
+      <c r="M8">
+        <v>20.79</v>
+      </c>
+      <c r="N8">
+        <v>9.01</v>
+      </c>
+      <c r="O8">
+        <v>17.52</v>
+      </c>
+      <c r="P8">
+        <v>12.57</v>
+      </c>
+      <c r="Q8">
+        <v>5.6</v>
+      </c>
+      <c r="R8">
+        <v>20</v>
+      </c>
+      <c r="S8">
+        <v>65.31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9">
+        <v>17.5</v>
+      </c>
+      <c r="D9">
+        <v>19.309999999999999</v>
+      </c>
+      <c r="E9">
+        <v>13.02</v>
+      </c>
+      <c r="F9">
+        <v>19.87</v>
+      </c>
+      <c r="G9">
+        <v>25.31</v>
+      </c>
+      <c r="H9">
+        <v>25.66</v>
+      </c>
+      <c r="I9">
+        <v>6</v>
+      </c>
+      <c r="J9">
+        <v>2.19</v>
+      </c>
+      <c r="K9">
+        <v>35</v>
+      </c>
+      <c r="L9">
+        <v>15</v>
+      </c>
+      <c r="M9">
+        <v>17.34</v>
+      </c>
+      <c r="N9">
+        <v>11.35</v>
+      </c>
+      <c r="O9">
+        <v>16.71</v>
+      </c>
+      <c r="P9">
+        <v>18.190000000000001</v>
+      </c>
+      <c r="Q9">
+        <v>8.2200000000000006</v>
+      </c>
+      <c r="R9">
+        <v>20</v>
+      </c>
+      <c r="S9">
+        <v>68.069999999999993</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10">
+        <v>20</v>
+      </c>
+      <c r="D10">
+        <v>22.18</v>
+      </c>
+      <c r="E10">
+        <v>13.86</v>
+      </c>
+      <c r="F10">
+        <v>949</v>
+      </c>
+      <c r="G10">
+        <v>27.5</v>
+      </c>
+      <c r="H10">
+        <v>37.24</v>
+      </c>
+      <c r="I10">
+        <v>7</v>
+      </c>
+      <c r="J10">
+        <v>0.2</v>
+      </c>
+      <c r="K10">
+        <v>28.72</v>
+      </c>
+      <c r="L10">
+        <v>15</v>
+      </c>
+      <c r="M10">
+        <v>13.37</v>
+      </c>
+      <c r="N10">
+        <v>12.31</v>
+      </c>
+      <c r="O10">
+        <v>19.47</v>
+      </c>
+      <c r="P10">
+        <v>22.7</v>
+      </c>
+      <c r="Q10">
+        <v>0.11</v>
+      </c>
+      <c r="R10">
+        <v>20</v>
+      </c>
+      <c r="S10">
+        <v>49.28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11">
+        <v>18.5</v>
+      </c>
+      <c r="D11">
+        <v>2777</v>
+      </c>
+      <c r="E11">
+        <v>17.37</v>
+      </c>
+      <c r="F11">
+        <v>14.6</v>
+      </c>
+      <c r="G11">
+        <v>27.28</v>
+      </c>
+      <c r="H11">
+        <v>27.04</v>
+      </c>
+      <c r="I11">
+        <v>2.5</v>
+      </c>
+      <c r="J11">
+        <v>2.66</v>
+      </c>
+      <c r="K11">
+        <v>33.89</v>
+      </c>
+      <c r="L11">
+        <v>15</v>
+      </c>
+      <c r="M11">
+        <v>15.2</v>
+      </c>
+      <c r="N11">
+        <v>12.46</v>
+      </c>
+      <c r="O11">
+        <v>5.07</v>
+      </c>
+      <c r="P11">
+        <v>18.53</v>
+      </c>
+      <c r="Q11">
+        <v>5.29</v>
+      </c>
+      <c r="R11">
+        <v>20</v>
+      </c>
+      <c r="S11">
+        <v>41.13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="52.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="70.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="19" width="8.7265625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>133</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CBE1785-8B4D-42A6-8DC3-3071B76D8AF9}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="51.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>